<commit_message>
Fix 2024E net income/EPS realism + add top-3 holders
- net income is annualized by a seasonality factor (soft Q4), NOT x4/3: FY2024E NI
  ₱10.6bn (was ₱13.5bn; matches the ~₱10.5bn full-year run-rate). Revenue/EBIT still x4/3,
  so the DCF fair value (₱27.35, NOPAT-based) is unchanged.
- EPS now on a common basis (deducts preferred dividends): ₱3.47→₱4.58, consistent with
  the filing's reported 9M EPS of ₱3.43
- front page: added Major shareholders (Trident 56.9% / public float / Ayala preferred)
- coverage-initiation note; 52-wk range relabeled estimated
- live Excel recalcs to the corrected NI/EPS; examples refreshed

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/mwc_model.xlsx
+++ b/examples/mwc_model.xlsx
@@ -1050,7 +1050,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B35"/>
+  <dimension ref="A1:B36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1254,7 +1254,7 @@
         </is>
       </c>
       <c r="B22" s="14" t="n">
-        <v>13470128</v>
+        <v>10607725.8</v>
       </c>
     </row>
     <row r="23">
@@ -1366,6 +1366,16 @@
       </c>
       <c r="B35" s="16" t="n">
         <v>22.36</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Preferred dividend (₱000/yr)</t>
+        </is>
+      </c>
+      <c r="B36" s="14" t="n">
+        <v>1600000</v>
       </c>
     </row>
   </sheetData>
@@ -1722,27 +1732,27 @@
         </is>
       </c>
       <c r="B14" s="9">
-        <f>B13*1000/Assumptions!$B$34</f>
+        <f>(B13-Assumptions!$B$36)*1000/Assumptions!$B$34</f>
         <v/>
       </c>
       <c r="C14" s="9">
-        <f>C13*1000/Assumptions!$B$34</f>
+        <f>(C13-Assumptions!$B$36)*1000/Assumptions!$B$34</f>
         <v/>
       </c>
       <c r="D14" s="9">
-        <f>D13*1000/Assumptions!$B$34</f>
+        <f>(D13-Assumptions!$B$36)*1000/Assumptions!$B$34</f>
         <v/>
       </c>
       <c r="E14" s="9">
-        <f>E13*1000/Assumptions!$B$34</f>
+        <f>(E13-Assumptions!$B$36)*1000/Assumptions!$B$34</f>
         <v/>
       </c>
       <c r="F14" s="9">
-        <f>F13*1000/Assumptions!$B$34</f>
+        <f>(F13-Assumptions!$B$36)*1000/Assumptions!$B$34</f>
         <v/>
       </c>
       <c r="G14" s="9">
-        <f>G13*1000/Assumptions!$B$34</f>
+        <f>(G13-Assumptions!$B$36)*1000/Assumptions!$B$34</f>
         <v/>
       </c>
     </row>

</xml_diff>